<commit_message>
Momentum scan results 2026-08-28
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_2026-08-28.xlsx
+++ b/results/momentum_failcodes_2026-08-28.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A514"/>
+  <dimension ref="A1:A523"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,637 +426,637 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ABLV</t>
+          <t>ABNB</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AARD</t>
+          <t>AD</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ABAT</t>
+          <t>BRNX</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AIRE</t>
+          <t>ACET</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ACHV</t>
+          <t>AIDX</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AIDX</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ALCO</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABTS</t>
+          <t>ATOS</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AWRE</t>
+          <t>ADAMK</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AMST</t>
+          <t>CGTL</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ACET</t>
+          <t>NXPL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ACU</t>
+          <t>ADBE</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BMRA</t>
+          <t>COYA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ATLX</t>
+          <t>OCCIN</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADAMH</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BNKK</t>
+          <t>DXST</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ADAMI</t>
+          <t>QNRX</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>AEI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BORR</t>
+          <t>ENGN</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ADAMN</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ELUT</t>
+          <t>AERT</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BSEM</t>
+          <t>FLD</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AEYE</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ERNA</t>
+          <t>FULC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CGTL</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ADVB</t>
+          <t>GAUZ</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AESP</t>
+          <t>AGPU</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FLD</t>
+          <t>GFAI</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CNTN</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>GUTS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>AIFA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>GSRV</t>
+          <t>IMPP</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DLPN</t>
+          <t>AIFC</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AIOS</t>
+          <t>IONS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AKTS</t>
+          <t>ALGS</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>HDRN</t>
+          <t>KLRS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DUKR</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AIRT</t>
+          <t>LEE</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LBTYA</t>
+          <t>LNZA</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ELVR</t>
+          <t>AMR</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>LUCD</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ALT</t>
+          <t>ANGO</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LBTYK</t>
+          <t>MFP</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>EVAX</t>
+          <t>ANGX</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ANAB</t>
+          <t>MODD</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ALVO</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PPIH</t>
+          <t>NAMM</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>EZRA</t>
+          <t>APLM</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>APPF</t>
+          <t>OPTX</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AMCX</t>
+          <t>APPF</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SERA</t>
+          <t>PPBT</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>FLUX</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>QSI</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>APRE</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FWRG</t>
+          <t>RECT</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AMR</t>
+          <t>AQST</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>RHLD</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>GFAI</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>ARCC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TH</t>
+          <t>SLDP</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>GRNQ</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>TH</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ANY</t>
+          <t>ARTNA</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GRRR</t>
+          <t>WHK</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>APGE</t>
+          <t>ASBP</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ISNR</t>
+          <t>ASMB</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>AYA</t>
+          <t>ATAT</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>APMC</t>
+          <t>ATKR</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LONA</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BCCQ</t>
+          <t>AUGO</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ARCL</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>OCGN</t>
+          <t>AXGN</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BIII</t>
+          <t>AYA</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ARCT</t>
+          <t>BANX</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PAVM</t>
+          <t>BBNX</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>BCRX</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ARGX</t>
+          <t>BEEP</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BLMN</t>
+          <t>BFRI</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ASUR</t>
+          <t>BGC</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PMEC</t>
+          <t>BHFAO</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>BIII</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>QTI</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BPYPN</t>
+          <t>BLSM</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AUGO</t>
+          <t>BMEA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RECT</t>
+          <t>BMNP</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BPYPO</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>AURA</t>
+          <t>BPYPN</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RYM</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
@@ -1077,2940 +1077,3003 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>BRR</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BRNX</t>
+          <t>BRZE</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>BSBK</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TLSA</t>
+          <t>BSVN</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>AZTR</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>BTBD</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BANX</t>
+          <t>BTCS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BGC</t>
+          <t>BTGO</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>BULL</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>BULLW</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>BIVI</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BWBBP</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>BYND</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>CACC</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CCG</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BLSM</t>
+          <t>CBAT</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CCU</t>
+          <t>CBLL</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>BMEA</t>
+          <t>CCCC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BMNP</t>
+          <t>CCSI</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CELU</t>
+          <t>CDLR</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>BPYPM</t>
+          <t>CDW</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CGBD</t>
+          <t>CEG</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>CELH</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CHEC</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BTBD</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CG</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>BTCS</t>
+          <t>CGAU</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CMMB</t>
+          <t>CGBD</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BTCT</t>
+          <t>CGEM</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CNOBP</t>
+          <t>CHEF</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>BTGO</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>COUR</t>
+          <t>CLBK</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BTLN</t>
+          <t>CLLS</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>BTOC</t>
+          <t>CMMB</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CSHR</t>
+          <t>CNDT</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BULLW</t>
+          <t>CNSP</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CYPH</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>BWIV</t>
+          <t>COCP</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>CAAS</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>CORT</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CABA</t>
+          <t>COUR</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>DFDV</t>
+          <t>CPB</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CADL</t>
+          <t>CPRT</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>DFDVW</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CARL</t>
+          <t>CRBP</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>CRNX</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CCEC</t>
+          <t>CRON</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>CSWC</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>CTNM</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>CTSH</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>EVER</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>CWBC</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>FBLA</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FORR</t>
+          <t>DERM</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CGAU</t>
+          <t>DHCNI</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CGEM</t>
+          <t>DJCO</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>FWDI</t>
+          <t>DMC</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>CGON</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>FWONA</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>CHCI</t>
+          <t>DSGN</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>CHNR</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CHSCL</t>
+          <t>DUOL</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GENVR</t>
+          <t>DXCM</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>CHSCO</t>
+          <t>ECPG</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HBIO</t>
+          <t>EDIT</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>CLBK</t>
+          <t>EDRY</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CNDT</t>
+          <t>ELBM</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>HLNE</t>
+          <t>ELE</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CNET</t>
+          <t>ELMT</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>HNST</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>CNR</t>
+          <t>EOLS</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>HSDT</t>
+          <t>EROK</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>ESEA</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>COCP</t>
+          <t>EXE</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>HYPD</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>EXFY</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>IDAI</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>COYA</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>FCBC</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>CRBP</t>
+          <t>FCFS</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>IPSC</t>
+          <t>FCNCO</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CRCT</t>
+          <t>FIVN</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>IVA</t>
+          <t>FLXS</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CSWC</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>KARO</t>
+          <t>FORR</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>CTNM</t>
+          <t>FRHC</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>KELYA</t>
+          <t>FRNM</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>KRNY</t>
+          <t>FSEA</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>KZIA</t>
+          <t>FSSL</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>DCBG</t>
+          <t>FTAIM</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>LASE</t>
+          <t>FVNNR</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>DEFT</t>
+          <t>GAIN</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>LEXX</t>
+          <t>GALT</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>DERM</t>
+          <t>GASS</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>LHSW</t>
+          <t>GCBC</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>GENK</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>DNUT</t>
+          <t>GENVR</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>LTGO</t>
+          <t>GEVO</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>DRMA</t>
+          <t>GLAD</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>GLBS</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>DUOT</t>
+          <t>GLIBA</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>MBINM</t>
+          <t>GLIBK</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>DWTX</t>
+          <t>GLNG</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>MDXG</t>
+          <t>GOLD</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>MESO</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>EDIT</t>
+          <t>GRML</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>METC</t>
+          <t>GRVY</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>GSHD</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>ELBM</t>
+          <t>GWAV</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>MOLN</t>
+          <t>GWRS</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>ELLA</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>HBANL</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>HBANM</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>ELVN</t>
+          <t>HBIO</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>EMBJ</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>EML</t>
+          <t>HELE</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>HELP</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>NA</t>
+          <t>HLNE</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>EU</t>
+          <t>HNST</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>NBRGU</t>
+          <t>HOWL</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>NBTX</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>NEO</t>
+          <t>HSIC</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>HSLV</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>NGEN</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>FBLG</t>
+          <t>HYMC</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>NKTX</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>FCBC</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>NMFC</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>FGII</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>IMC</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>NVA</t>
+          <t>IMRN</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>FLXS</t>
+          <t>INBX</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>INCY</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>FORTY</t>
+          <t>INO</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>OESX</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>OFS</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>FSHP</t>
+          <t>IOND</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>OGI</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>FSSL</t>
+          <t>IPEX</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>OMDA</t>
+          <t>IPHA</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>OMSE</t>
+          <t>IPVV</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>GAINZ</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>ORMP</t>
+          <t>ITIC</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>GASS</t>
+          <t>IVVD</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>OVID</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>GCBC</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>JG</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>PANL</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>GEMI</t>
+          <t>JSM</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>PBLS</t>
+          <t>KARO</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>KELYA</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>GLBS</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>GLE</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>PMTW</t>
+          <t>KMB</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>GLIBK</t>
+          <t>KMDA</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>PRE</t>
+          <t>KRNY</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>GLSI</t>
+          <t>KSPI</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>PRQR</t>
+          <t>KTTA</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>GMTL</t>
+          <t>KWY</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>PSNYW</t>
+          <t>KYMR</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>GRI</t>
+          <t>KYNB</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>PSUS</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>GROW</t>
+          <t>LBRX</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>GSHD</t>
+          <t>LCLN</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>PTN</t>
+          <t>LECO</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>GWRS</t>
+          <t>LEGH</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>HAIN</t>
+          <t>LEXX</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>RDI</t>
+          <t>LHSW</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>HELP</t>
+          <t>LIEN</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>RDVT</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>HGBL</t>
+          <t>LMRI</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>RILYG</t>
+          <t>LOPE</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>HHS</t>
+          <t>LTGO</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>RILYN</t>
+          <t>LXEO</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>HMR</t>
+          <t>LYFT</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>RILYZ</t>
+          <t>MCHX</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>HNRG</t>
+          <t>MDXG</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>RMNI</t>
+          <t>MELI</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>MENS</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>HQI</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>MEVO</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>HRMY</t>
+          <t>MFIN</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>HSCS</t>
+          <t>MGTX</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>SABR</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>HSLV</t>
+          <t>MLAB</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>SAGU</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>MTC</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>MTVA</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>SAV</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>MYSE</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>MYSZ</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>NAKA</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>NAVI</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>SIND</t>
+          <t>NCNO</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>IKT</t>
+          <t>NCT</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>SLDB</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>IMMR</t>
+          <t>NESR</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>SLMBP</t>
+          <t>NGEN</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>IMXI</t>
+          <t>NGNE</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>INCY</t>
+          <t>NHPAP</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>SMCIP</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>SOPH</t>
+          <t>NICM</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>IOND</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>NKTX</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>IPWR</t>
+          <t>NMFC</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>IQMX</t>
+          <t>NMFCZ</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>NRC</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>STDN</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>NSAIU</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>STHO</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>KEQU</t>
+          <t>NTLA</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>STKE</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>KEYY</t>
+          <t>NTRSO</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>NUTX</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>STRD</t>
+          <t>NVA</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>KIDZ</t>
+          <t>NVCT</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>STRF</t>
+          <t>NWGL</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>KMDA</t>
+          <t>NWSA</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>TAOX</t>
+          <t>OCCI</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>KRSP</t>
+          <t>OFS</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>TARS</t>
+          <t>OGI</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>OMDA</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>TAYD</t>
+          <t>OPCH</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>KSPI</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>KTTA</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>TIL</t>
+          <t>ORBS</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>ORIO</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>ORMP</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>TRNI</t>
+          <t>OVLY</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>LBRX</t>
+          <t>OXLC</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>USDE</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>LEGH</t>
+          <t>PANL</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>USDEW</t>
+          <t>PAYX</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>VCTR</t>
+          <t>PBM</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>LIEN</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>VGNT</t>
+          <t>PEGA</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>PEPG</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>VIR</t>
+          <t>PMTS</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>LILAP</t>
+          <t>PPC</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>WSE</t>
+          <t>PPHC</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>LIME</t>
+          <t>PPIH</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>LNSR</t>
+          <t>PRAA</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>LOPE</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>LPSN</t>
+          <t>PRDO</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>LUCY</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>PROK</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>PROV</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>MCGA</t>
+          <t>PRTA</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>MELI</t>
+          <t>PRZO</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>MENS</t>
+          <t>PSEC</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PSUS</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>MESH</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>MEVO</t>
+          <t>PXLW</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>MF</t>
+          <t>PYXS</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>MICC</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>MINE</t>
+          <t>QNCX</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>MLAB</t>
+          <t>RANI</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>MNOV</t>
+          <t>RAPP</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>MNSB</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>MSBIP</t>
+          <t>RCMT</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>MYSZ</t>
+          <t>RDVT</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>NAKA</t>
+          <t>RDZN</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>NAVI</t>
+          <t>REFI</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>NCT</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>NEOG</t>
+          <t>RENX</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>NEOV</t>
+          <t>RGLD</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>NEXM</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>NGNE</t>
+          <t>RILYN</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>NHPBP</t>
+          <t>RMBI</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>NICM</t>
+          <t>RMNI</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>NMFCZ</t>
+          <t>RMTI</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>NSTS</t>
+          <t>RNAC</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>RNXT</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>NVCR</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>NXPL</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>OCCI</t>
+          <t>RUM</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>OCLTU</t>
+          <t>RWAY</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>OGC</t>
+          <t>RZLV</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>ONBPO</t>
+          <t>SABR</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>ONCH</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>ORBS</t>
+          <t>SAV</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>ORIO</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>OTLY</t>
+          <t>SBC</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>SBFG</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>OXLC</t>
+          <t>SBLK</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>PACH</t>
+          <t>SBMT</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>PBAM</t>
+          <t>SCWO</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>SCZM</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>PLMK</t>
+          <t>SEGG</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>PNRG</t>
+          <t>SEIC</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>PPHC</t>
+          <t>SENEA</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>PRAA</t>
+          <t>SGHT</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>SGML</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>SHIM</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>PROV</t>
+          <t>SHIP</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>PRPO</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>PUSA</t>
+          <t>SLMBP</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>PYPD</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>QMCO</t>
+          <t>SLNG</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>QNCX</t>
+          <t>SLNHP</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>QRHC</t>
+          <t>SMCIP</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>QTTB</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>RACD</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>RCKT</t>
+          <t>SRPT</t>
         </is>
       </c>
     </row>
     <row r="415">
       <c r="A415" t="inlineStr">
         <is>
-          <t>REFI</t>
+          <t>SRRK</t>
         </is>
       </c>
     </row>
     <row r="416">
       <c r="A416" t="inlineStr">
         <is>
-          <t>REGCO</t>
+          <t>SSMR</t>
         </is>
       </c>
     </row>
     <row r="417">
       <c r="A417" t="inlineStr">
         <is>
-          <t>REGCP</t>
+          <t>SSNC</t>
         </is>
       </c>
     </row>
     <row r="418">
       <c r="A418" t="inlineStr">
         <is>
-          <t>RENX</t>
+          <t>STEP</t>
         </is>
       </c>
     </row>
     <row r="419">
       <c r="A419" t="inlineStr">
         <is>
-          <t>RFAI</t>
+          <t>STOK</t>
         </is>
       </c>
     </row>
     <row r="420">
       <c r="A420" t="inlineStr">
         <is>
-          <t>RGEN</t>
+          <t>STRA</t>
         </is>
       </c>
     </row>
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>RGLD</t>
+          <t>STRC</t>
         </is>
       </c>
     </row>
     <row r="422">
       <c r="A422" t="inlineStr">
         <is>
-          <t>RHLD</t>
+          <t>STRF</t>
         </is>
       </c>
     </row>
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>STRK</t>
         </is>
       </c>
     </row>
     <row r="424">
       <c r="A424" t="inlineStr">
         <is>
-          <t>RLYB</t>
+          <t>STTK</t>
         </is>
       </c>
     </row>
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>RMCO</t>
+          <t>SUNC</t>
         </is>
       </c>
     </row>
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>RWAY</t>
+          <t>SVRN</t>
         </is>
       </c>
     </row>
     <row r="427">
       <c r="A427" t="inlineStr">
         <is>
-          <t>RWAYI</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="428">
       <c r="A428" t="inlineStr">
         <is>
-          <t>RYOJ</t>
+          <t>SWVL</t>
         </is>
       </c>
     </row>
     <row r="429">
       <c r="A429" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>SY</t>
         </is>
       </c>
     </row>
     <row r="430">
       <c r="A430" t="inlineStr">
         <is>
-          <t>SAIH</t>
+          <t>TBPH</t>
         </is>
       </c>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>TEAM</t>
         </is>
       </c>
     </row>
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>SBFG</t>
+          <t>TII</t>
         </is>
       </c>
     </row>
     <row r="433">
       <c r="A433" t="inlineStr">
         <is>
-          <t>SBMT</t>
+          <t>TJGC</t>
         </is>
       </c>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
         <is>
-          <t>SCSC</t>
+          <t>TMC</t>
         </is>
       </c>
     </row>
     <row r="435">
       <c r="A435" t="inlineStr">
         <is>
-          <t>SCWO</t>
+          <t>TMCI</t>
         </is>
       </c>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
         <is>
-          <t>SCZM</t>
+          <t>TONT</t>
         </is>
       </c>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
         <is>
-          <t>SDGR</t>
+          <t>TOP</t>
         </is>
       </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
         <is>
-          <t>SENEA</t>
+          <t>TORO</t>
         </is>
       </c>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
         <is>
-          <t>SGHT</t>
+          <t>TPCS</t>
         </is>
       </c>
     </row>
     <row r="440">
       <c r="A440" t="inlineStr">
         <is>
-          <t>SGML</t>
+          <t>TPG</t>
         </is>
       </c>
     </row>
     <row r="441">
       <c r="A441" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>SHOT</t>
+          <t>TRIN</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>TRMD</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>TRNZ</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>SLP</t>
+          <t>TRON</t>
         </is>
       </c>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>USAU</t>
         </is>
       </c>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
         <is>
-          <t>SRTS</t>
+          <t>USDE</t>
         </is>
       </c>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>SSMR</t>
+          <t>VCTR</t>
         </is>
       </c>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
         <is>
-          <t>STEP</t>
+          <t>VGNT</t>
         </is>
       </c>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
         <is>
-          <t>STOK</t>
+          <t>VIR</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>STRZ</t>
+          <t>VOXR</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>STTK</t>
+          <t>VSNT</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>SUNC</t>
+          <t>WW</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>SVRN</t>
+          <t>XMAX</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>SY</t>
+          <t>XRN</t>
         </is>
       </c>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
         <is>
-          <t>TASK</t>
+          <t>ZSTK</t>
         </is>
       </c>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
         <is>
-          <t>TCBIO</t>
+          <t>BTCT</t>
         </is>
       </c>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
         <is>
-          <t>TGTX</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
         <is>
-          <t>TII</t>
+          <t>LOT</t>
         </is>
       </c>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
         <is>
-          <t>TJGC</t>
+          <t>GEN</t>
         </is>
       </c>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
         <is>
-          <t>TLF</t>
+          <t>SUPX</t>
         </is>
       </c>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
         <is>
-          <t>TOP</t>
+          <t>RACD</t>
         </is>
       </c>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>CHRS</t>
         </is>
       </c>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
         <is>
-          <t>USAU</t>
+          <t>MF</t>
         </is>
       </c>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
         <is>
-          <t>VOGX</t>
+          <t>RFAI</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>ACTU</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>WW</t>
+          <t>HHS</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>XMAX</t>
+          <t>AZTR</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>XRN</t>
+          <t>BLSH</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>XZO</t>
+          <t>DFDVW</t>
         </is>
       </c>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>NWGL</t>
+          <t>HDRN</t>
         </is>
       </c>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
         <is>
-          <t>BDSX</t>
+          <t>TAOX</t>
         </is>
       </c>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
         <is>
-          <t>SWVL</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>INMB</t>
+          <t>VOGX</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>IXHL</t>
+          <t>BNKK</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>CSTL</t>
+          <t>FWDI</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>AQST</t>
+          <t>RDI</t>
         </is>
       </c>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
         <is>
-          <t>CGEN</t>
+          <t>GLSI</t>
         </is>
       </c>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>SUJA</t>
         </is>
       </c>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
         <is>
-          <t>IMMX</t>
+          <t>OESX</t>
         </is>
       </c>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
         <is>
-          <t>MRKR</t>
+          <t>PACB</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>BEEP</t>
+          <t>CYPH</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>CHTRP</t>
+          <t>CABA</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>GALT</t>
+          <t>CAN</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>PBM</t>
+          <t>METC</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>CLPS</t>
+          <t>BCDA</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>COPR</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>EOLS</t>
+          <t>CARL</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>IDYA</t>
+          <t>IBG</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>GAUZ</t>
+          <t>HYPD</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>FCUV</t>
+          <t>DAIC</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>SUPX</t>
+          <t>HNRG</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>BANL</t>
+          <t>ARCT</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>ODTX</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>ACB</t>
+          <t>HSCS</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>NEXT</t>
+          <t>BANL</t>
         </is>
       </c>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>HITI</t>
+          <t>USDEW</t>
         </is>
       </c>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
         <is>
-          <t>ZSTK</t>
+          <t>PRE</t>
         </is>
       </c>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
         <is>
-          <t>STRK</t>
+          <t>BIVI</t>
         </is>
       </c>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
         <is>
-          <t>MTC</t>
+          <t>GLE</t>
         </is>
       </c>
     </row>
     <row r="501">
       <c r="A501" t="inlineStr">
         <is>
-          <t>BCDA</t>
+          <t>IXHL</t>
         </is>
       </c>
     </row>
     <row r="502">
       <c r="A502" t="inlineStr">
         <is>
-          <t>KYNB</t>
+          <t>CNR</t>
         </is>
       </c>
     </row>
     <row r="503">
       <c r="A503" t="inlineStr">
         <is>
-          <t>NVCT</t>
+          <t>EU</t>
         </is>
       </c>
     </row>
     <row r="504">
       <c r="A504" t="inlineStr">
         <is>
-          <t>NERV</t>
+          <t>FBLG</t>
         </is>
       </c>
     </row>
     <row r="505">
       <c r="A505" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>CELU</t>
         </is>
       </c>
     </row>
     <row r="506">
       <c r="A506" t="inlineStr">
         <is>
-          <t>DTCX</t>
+          <t>GRI</t>
         </is>
       </c>
     </row>
     <row r="507">
       <c r="A507" t="inlineStr">
         <is>
-          <t>INBX</t>
+          <t>SBET</t>
         </is>
       </c>
     </row>
     <row r="508">
       <c r="A508" t="inlineStr">
         <is>
-          <t>XXI</t>
+          <t>DFDV</t>
         </is>
       </c>
     </row>
     <row r="509">
       <c r="A509" t="inlineStr">
         <is>
-          <t>JANX</t>
+          <t>ALVO</t>
         </is>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="inlineStr">
         <is>
-          <t>IBG</t>
+          <t>CADL</t>
         </is>
       </c>
     </row>
     <row r="511">
       <c r="A511" t="inlineStr">
         <is>
-          <t>SRRK</t>
+          <t>CPIX</t>
         </is>
       </c>
     </row>
     <row r="512">
       <c r="A512" t="inlineStr">
         <is>
-          <t>ACTU</t>
+          <t>EML</t>
         </is>
       </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>CENN</t>
+          <t>MRKR</t>
         </is>
       </c>
     </row>
     <row r="514">
       <c r="A514" t="inlineStr">
         <is>
-          <t>TRON</t>
+          <t>CRML</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>CDZI</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>PGY</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>SPRB</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>ACFN</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>DEFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>AIRE</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>IQMX</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>DTCX</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>FGNX</t>
         </is>
       </c>
     </row>

</xml_diff>